<commit_message>
Updated Excel on 1st June
New Report
</commit_message>
<xml_diff>
--- a/Students_Final.xlsx
+++ b/Students_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/swapnilbaranwal/Desktop/Friends LIbrary Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA34F08-D222-8D4A-802C-DF34D4A87D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88CA2A1-485B-A148-9BF3-1B7C8C40AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="50">
   <si>
     <t>S.No.</t>
   </si>
@@ -166,7 +166,10 @@
     <t>Paid</t>
   </si>
   <si>
-    <t>Unpaid</t>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>Prashant</t>
   </si>
 </sst>
 </file>
@@ -589,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -778,7 +781,7 @@
         <v>47</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -934,7 +937,9 @@
       <c r="E8" s="5">
         <v>700</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="2">
+        <v>43</v>
+      </c>
       <c r="G8" s="6" t="s">
         <v>21</v>
       </c>
@@ -947,7 +952,9 @@
       <c r="J8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -974,13 +981,21 @@
         <v>700</v>
       </c>
       <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="G9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="J9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="7"/>
+      <c r="K9" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
@@ -1710,7 +1725,7 @@
         <v>47</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -1807,9 +1822,142 @@
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
     </row>
+    <row r="29" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="4">
+        <v>46170</v>
+      </c>
+      <c r="E29" s="5">
+        <v>700</v>
+      </c>
+      <c r="F29" s="2">
+        <v>13</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
+      <c r="S29" s="2"/>
+    </row>
+    <row r="30" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="4">
+        <v>46174</v>
+      </c>
+      <c r="E30" s="5">
+        <v>700</v>
+      </c>
+      <c r="F30" s="2">
+        <v>50</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+    </row>
+    <row r="31" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="4">
+        <v>46174</v>
+      </c>
+      <c r="E31" s="5">
+        <v>700</v>
+      </c>
+      <c r="F31" s="2">
+        <v>49</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
+      <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
+      <c r="S31" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G9 G10 H9 H10 I4 I9 I10 I26 J2 J4 J6 J9 J10 J11 J13 J14 J17 J19 J21 J22 J23 J24 J25 J26 K2 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 L2 L3 L4 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 M2 M3 M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 N2 N3 N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 O2 O3 O4 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 P2 P3 P4 P5 P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 Q2 Q3 Q4 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 R2 R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 S2 S3 S4 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L2:S31 I26 J2 I4:J4 J6 J9:J11 J13:J14 J17 J19 J21:J26 G10:I10 K2:K8 K10:K29" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Paid,Unpaid"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>